<commit_message>
added assembly and tweaked parameters for correct fit.
</commit_message>
<xml_diff>
--- a/calculations/D38999_26AXXXX_Dimensions.xlsx
+++ b/calculations/D38999_26AXXXX_Dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lelem\git_repositories\projects\D38999-3MF\calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1516BB6A-23B3-48F6-8A83-4022DCD8A1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0742377-26B7-42F7-8255-F8C68AA24260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{58E9E39D-3151-410B-8DC1-39983DB63DF0}"/>
+    <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12336" xr2:uid="{58E9E39D-3151-410B-8DC1-39983DB63DF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -467,12 +467,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -811,6 +810,34 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="15.578125" customWidth="1"/>
+    <col min="2" max="3" width="28.3671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.15625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.1015625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.1015625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.20703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.47265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.9453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.26171875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.26171875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.9453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.9453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.83984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.9453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.68359375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="26.62890625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.1015625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="28.3671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.83984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="37.15625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.1015625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.1015625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.9453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="28.47265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="29.9453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.47265625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="27.05078125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.55000000000000004">
@@ -888,25 +915,25 @@
       <c r="W2" t="s">
         <v>116</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" t="s">
         <v>104</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Y2" t="s">
         <v>34</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="Z2" t="s">
         <v>43</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AA2" t="s">
         <v>44</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AB2" t="s">
         <v>40</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AC2" t="s">
         <v>36</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AD2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -980,25 +1007,25 @@
       <c r="W3">
         <v>1.32</v>
       </c>
-      <c r="X3" s="4">
+      <c r="X3">
         <v>10</v>
       </c>
-      <c r="Y3" s="4">
+      <c r="Y3">
         <v>0.5</v>
       </c>
-      <c r="Z3" s="4">
+      <c r="Z3">
         <v>1</v>
       </c>
-      <c r="AA3" s="4">
+      <c r="AA3">
         <v>5</v>
       </c>
-      <c r="AB3" s="4">
+      <c r="AB3">
         <v>5</v>
       </c>
-      <c r="AC3" s="4">
+      <c r="AC3">
         <v>4</v>
       </c>
-      <c r="AD3" s="4">
+      <c r="AD3">
         <v>31</v>
       </c>
     </row>

</xml_diff>